<commit_message>
chore: consolidate game into index.html and refresh unit values
- Move primary entry to root index.html with split css/style.css
- Remove legacy source/audio/backup copies no longer used
- Add latest unit attribute sheet 20260730.xlsx
- Ignore agent memory and slide-build artifacts
</commit_message>
<xml_diff>
--- a/单位属性表/20260726.xlsx
+++ b/单位属性表/20260726.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cruelworld\Desktop\小游戏\奇境王冠\单位属性表\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FE53561-86FF-44AC-9B56-667BBEBFD839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{142A9238-1AC4-4D1F-A5A1-298602F3DF5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13986" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="70">
   <si>
     <t>单位</t>
   </si>
@@ -664,6 +664,18 @@
   </si>
   <si>
     <t>随机强化其中一种单位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ai加农炮使用策略：</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>当检测到某一路的威胁值高于一定值时，ai会停止购买棋子，攒钱买加农炮</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>棋子通过药水变大后，攻击距离同步变大相同百分比</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -671,7 +683,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <name val="Microsoft YaHei"/>
@@ -775,8 +787,14 @@
       <family val="2"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -849,6 +867,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -888,7 +912,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -929,6 +953,15 @@
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -950,6 +983,9 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -959,7 +995,10 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1301,7 +1340,8 @@
   <cols>
     <col min="1" max="1" width="17.3125" style="5" customWidth="1"/>
     <col min="2" max="5" width="14" style="5" customWidth="1"/>
-    <col min="6" max="7" width="12" style="5" customWidth="1"/>
+    <col min="6" max="6" width="12" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14.7890625" style="5" customWidth="1"/>
     <col min="8" max="8" width="16.05078125" style="5" customWidth="1"/>
     <col min="9" max="11" width="25.47265625" style="5" customWidth="1"/>
     <col min="12" max="12" width="20" style="5" customWidth="1"/>
@@ -1483,10 +1523,10 @@
         <v>10</v>
       </c>
       <c r="C5" s="2">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="D5" s="2">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E5" s="2">
         <v>50</v>
@@ -1514,22 +1554,22 @@
       </c>
       <c r="M5" s="6">
         <f>D5/G5*1000</f>
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:14" s="6" customFormat="1"/>
     <row r="7" spans="1:14" s="6" customFormat="1"/>
     <row r="8" spans="1:14" s="6" customFormat="1"/>
     <row r="9" spans="1:14" ht="46">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
       <c r="H9" s="12" t="s">
         <v>61</v>
       </c>
@@ -1543,17 +1583,17 @@
       <c r="N9" s="6"/>
     </row>
     <row r="10" spans="1:14" ht="20">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="15">
+      <c r="B10" s="23"/>
+      <c r="C10" s="18">
         <v>5</v>
       </c>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
       <c r="H10" s="13" t="s">
         <v>63</v>
       </c>
@@ -1567,17 +1607,17 @@
       <c r="N10" s="6"/>
     </row>
     <row r="11" spans="1:14" ht="19.350000000000001">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16">
+      <c r="B11" s="19"/>
+      <c r="C11" s="19">
         <v>20</v>
       </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
@@ -1587,19 +1627,21 @@
       <c r="N11" s="6"/>
     </row>
     <row r="12" spans="1:14" ht="19.350000000000001">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16">
+      <c r="B12" s="19"/>
+      <c r="C12" s="19">
         <v>40</v>
       </c>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" s="29"/>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
@@ -1705,7 +1747,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:14" s="6" customFormat="1" ht="48">
+    <row r="17" spans="1:14" s="6" customFormat="1" ht="32">
       <c r="A17" s="11" t="s">
         <v>57</v>
       </c>
@@ -1743,10 +1785,10 @@
       <c r="N18" s="6"/>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="24">
+      <c r="B19" s="14">
         <v>15</v>
       </c>
       <c r="C19" s="6"/>
@@ -1830,18 +1872,22 @@
       <c r="M23" s="6"/>
       <c r="N23" s="6"/>
     </row>
-    <row r="24" spans="1:14" ht="28">
-      <c r="A24" s="17" t="s">
+    <row r="24" spans="1:14" ht="35" customHeight="1">
+      <c r="A24" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="G24" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="H24" s="24"/>
+      <c r="I24" s="15"/>
       <c r="J24" s="6"/>
       <c r="K24" s="6"/>
       <c r="L24" s="6"/>
@@ -1852,131 +1898,131 @@
       <c r="A25" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
     </row>
     <row r="26" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A26" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
     </row>
     <row r="27" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19">
+      <c r="B27" s="22"/>
+      <c r="C27" s="22">
         <v>20</v>
       </c>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
     </row>
     <row r="28" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A28" s="19" t="s">
+      <c r="A28" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19">
+      <c r="B28" s="22"/>
+      <c r="C28" s="22">
         <v>20</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
     </row>
     <row r="29" spans="1:14" s="6" customFormat="1" ht="16">
-      <c r="A29" s="19" t="s">
+      <c r="A29" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19">
+      <c r="B29" s="22"/>
+      <c r="C29" s="22">
         <v>1000</v>
       </c>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
     </row>
     <row r="30" spans="1:14" s="6" customFormat="1" ht="28">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
     </row>
     <row r="31" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A31" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
     </row>
     <row r="32" spans="1:14" s="6" customFormat="1" ht="16">
       <c r="A32" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
     </row>
     <row r="33" spans="1:5" s="6" customFormat="1" ht="16">
-      <c r="A33" s="19" t="s">
+      <c r="A33" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19">
+      <c r="B33" s="22"/>
+      <c r="C33" s="22">
         <v>2000</v>
       </c>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
     </row>
     <row r="34" spans="1:5" s="6" customFormat="1" ht="16">
-      <c r="A34" s="19" t="s">
+      <c r="A34" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="19"/>
-      <c r="C34" s="19">
+      <c r="B34" s="22"/>
+      <c r="C34" s="22">
         <v>150</v>
       </c>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
     </row>
     <row r="35" spans="1:5" s="6" customFormat="1" ht="44" customHeight="1">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="B35" s="21"/>
-      <c r="C35" s="22" t="s">
+      <c r="B35" s="25"/>
+      <c r="C35" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="26"/>
     </row>
     <row r="36" spans="1:5" s="6" customFormat="1">
-      <c r="A36" s="23" t="s">
+      <c r="A36" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="23"/>
-      <c r="C36" s="23" t="s">
+      <c r="B36" s="27"/>
+      <c r="C36" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="D36" s="23"/>
-      <c r="E36" s="23"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
     </row>
     <row r="37" spans="1:5" s="6" customFormat="1"/>
     <row r="38" spans="1:5" s="6" customFormat="1"/>
@@ -1995,7 +2041,7 @@
     <row r="51" s="6" customFormat="1"/>
     <row r="52" s="6" customFormat="1"/>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="29">
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="C34:E34"/>
     <mergeCell ref="A35:B35"/>
@@ -2023,6 +2069,8 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="C12:G12"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="H12:I12"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>